<commit_message>
Add A1 corpus cleaning notebook and produce corpus.json
- Built A1_corpus_cleaning.ipynb: loads Excel metadata, normalizes text, outputs corpus.json
- 167 songs, each with a single `text` field (translated version for songs 023, 061, 138)
- Added tests/test_corpus.py with 10 passing tests
- Updated project-plan.md: documents resolved data issues and translation approach
</commit_message>
<xml_diff>
--- a/songs/songs_summary.xlsx
+++ b/songs/songs_summary.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b29335a1de609aeb/Desktop/מיני פרויקט שלמה ארצי/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sap-my.sharepoint.com/personal/yuval_sadot_sap_com/Documents/Documents/School/MINI/songs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="39" documentId="8_{AB6D7C70-1778-461B-9270-A14BF7B5CECE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{12ACD060-2CA2-41C5-8AD6-E1BEE0288C22}"/>
+  <xr:revisionPtr revIDLastSave="47" documentId="8_{AB6D7C70-1778-461B-9270-A14BF7B5CECE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3880B829-D6FA-734D-99A4-CA28B5B4811A}"/>
   <bookViews>
-    <workbookView xWindow="1520" yWindow="1520" windowWidth="14400" windowHeight="7270" xr2:uid="{22D40CF9-48C2-4438-BAF2-71908CEA5B3A}"/>
+    <workbookView xWindow="1520" yWindow="1520" windowWidth="17200" windowHeight="8780" xr2:uid="{22D40CF9-48C2-4438-BAF2-71908CEA5B3A}"/>
   </bookViews>
   <sheets>
     <sheet name="גיליון1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="339" uniqueCount="175">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="339" uniqueCount="174">
   <si>
     <t>title</t>
   </si>
@@ -268,15 +268,9 @@
     <t>האם השלישית</t>
   </si>
   <si>
-    <t>אנחנו לא צריכים</t>
-  </si>
-  <si>
     <t>תפילת ערבית</t>
   </si>
   <si>
-    <t>הבלדה על לבן בן בתואל</t>
-  </si>
-  <si>
     <t>ירח</t>
   </si>
   <si>
@@ -535,9 +529,6 @@
     <t>הייתי והיינו</t>
   </si>
   <si>
-    <t>Love לאהבה</t>
-  </si>
-  <si>
     <t>הריקוד האחרון של 1956</t>
   </si>
   <si>
@@ -553,13 +544,19 @@
     <t>המזדנבות</t>
   </si>
   <si>
-    <t>נחל ים</t>
-  </si>
-  <si>
     <t>שיר קיץ</t>
   </si>
   <si>
-    <t>אהבתיה</t>
+    <t>יותר מזה אנחנו לא צריכים</t>
+  </si>
+  <si>
+    <t>בלדה על לבן בן בתואל</t>
+  </si>
+  <si>
+    <t>נח״ל ים</t>
+  </si>
+  <si>
+    <t>פתאום עכשיו פתאום היום</t>
   </si>
 </sst>
 </file>
@@ -570,7 +567,7 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <charset val="177"/>
       <scheme val="minor"/>
@@ -579,13 +576,13 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="8"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <charset val="177"/>
       <scheme val="minor"/>
@@ -737,6 +734,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1050,15 +1051,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27F6E413-9FD9-4B97-99D0-4DECF06B448E}">
   <dimension ref="A1:D168"/>
-  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="12.75" customWidth="1"/>
-    <col min="2" max="2" width="27.25" customWidth="1"/>
+    <col min="1" max="1" width="12.6640625" customWidth="1"/>
+    <col min="2" max="2" width="27.1640625" customWidth="1"/>
     <col min="3" max="3" width="29.1640625" customWidth="1"/>
     <col min="4" max="4" width="49.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>3</v>
       </c>
@@ -1072,7 +1073,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" s="4">
         <v>1</v>
       </c>
@@ -1086,7 +1087,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" s="4">
         <v>2</v>
       </c>
@@ -1100,7 +1101,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" s="4">
         <v>3</v>
       </c>
@@ -1114,7 +1115,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" s="4">
         <v>4</v>
       </c>
@@ -1128,7 +1129,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" s="4">
         <v>5</v>
       </c>
@@ -1142,7 +1143,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" s="4">
         <v>6</v>
       </c>
@@ -1156,12 +1157,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" s="4">
         <v>7</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="C8" s="4">
         <v>2025</v>
@@ -1170,7 +1171,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9" s="4">
         <v>8</v>
       </c>
@@ -1184,7 +1185,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" s="4">
         <v>9</v>
       </c>
@@ -1198,7 +1199,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11" s="4">
         <v>10</v>
       </c>
@@ -1212,7 +1213,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A12" s="4">
         <v>11</v>
       </c>
@@ -1226,7 +1227,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A13" s="4">
         <v>12</v>
       </c>
@@ -1240,7 +1241,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A14" s="4">
         <v>13</v>
       </c>
@@ -1254,7 +1255,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A15" s="4">
         <v>14</v>
       </c>
@@ -1268,7 +1269,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A16" s="4">
         <v>15</v>
       </c>
@@ -1282,7 +1283,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" s="2">
         <v>16</v>
       </c>
@@ -1296,7 +1297,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18" s="2">
         <v>17</v>
       </c>
@@ -1310,7 +1311,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19" s="2">
         <v>18</v>
       </c>
@@ -1324,7 +1325,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20" s="2">
         <v>19</v>
       </c>
@@ -1338,7 +1339,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A21" s="2">
         <v>20</v>
       </c>
@@ -1352,7 +1353,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A22" s="2">
         <v>21</v>
       </c>
@@ -1366,7 +1367,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A23" s="2">
         <v>22</v>
       </c>
@@ -1380,7 +1381,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A24" s="2">
         <v>23</v>
       </c>
@@ -1394,7 +1395,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A25" s="2">
         <v>24</v>
       </c>
@@ -1408,12 +1409,12 @@
         <v>18</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A26" s="2">
         <v>25</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="C26" s="2">
         <v>2016</v>
@@ -1422,7 +1423,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A27" s="2">
         <v>26</v>
       </c>
@@ -1436,7 +1437,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A28" s="2">
         <v>27</v>
       </c>
@@ -1450,7 +1451,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A29" s="2">
         <v>28</v>
       </c>
@@ -1464,7 +1465,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A30" s="2">
         <v>29</v>
       </c>
@@ -1478,7 +1479,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A31" s="3">
         <v>30</v>
       </c>
@@ -1492,7 +1493,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A32" s="3">
         <v>31</v>
       </c>
@@ -1506,7 +1507,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A33" s="3">
         <v>32</v>
       </c>
@@ -1520,7 +1521,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A34" s="3">
         <v>33</v>
       </c>
@@ -1534,7 +1535,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A35" s="3">
         <v>34</v>
       </c>
@@ -1548,7 +1549,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A36" s="3">
         <v>35</v>
       </c>
@@ -1562,7 +1563,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A37" s="3">
         <v>36</v>
       </c>
@@ -1576,7 +1577,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A38" s="3">
         <v>37</v>
       </c>
@@ -1590,7 +1591,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A39" s="3">
         <v>38</v>
       </c>
@@ -1604,7 +1605,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A40" s="3">
         <v>39</v>
       </c>
@@ -1618,7 +1619,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A41" s="3">
         <v>40</v>
       </c>
@@ -1632,12 +1633,12 @@
         <v>32</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A42" s="3">
         <v>41</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="C42" s="3">
         <v>2012</v>
@@ -1646,7 +1647,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A43" s="4">
         <v>42</v>
       </c>
@@ -1660,7 +1661,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A44" s="4">
         <v>43</v>
       </c>
@@ -1674,7 +1675,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A45" s="4">
         <v>44</v>
       </c>
@@ -1688,12 +1689,12 @@
         <v>43</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A46" s="4">
         <v>45</v>
       </c>
       <c r="B46" s="4" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C46" s="4">
         <v>2007</v>
@@ -1702,7 +1703,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A47" s="4">
         <v>46</v>
       </c>
@@ -1716,7 +1717,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A48" s="4">
         <v>47</v>
       </c>
@@ -1730,7 +1731,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A49" s="4">
         <v>48</v>
       </c>
@@ -1744,7 +1745,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A50" s="4">
         <v>49</v>
       </c>
@@ -1758,7 +1759,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A51" s="4">
         <v>50</v>
       </c>
@@ -1772,7 +1773,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A52" s="4">
         <v>51</v>
       </c>
@@ -1786,12 +1787,12 @@
         <v>43</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A53" s="4">
         <v>52</v>
       </c>
       <c r="B53" s="4" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="C53" s="4">
         <v>2007</v>
@@ -1800,7 +1801,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A54" s="4">
         <v>53</v>
       </c>
@@ -1814,7 +1815,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A55" s="4">
         <v>54</v>
       </c>
@@ -1828,7 +1829,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A56" s="4">
         <v>55</v>
       </c>
@@ -1842,7 +1843,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A57" s="4">
         <v>56</v>
       </c>
@@ -1856,7 +1857,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A58" s="2">
         <v>57</v>
       </c>
@@ -1870,7 +1871,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A59" s="2">
         <v>58</v>
       </c>
@@ -1884,7 +1885,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A60" s="2">
         <v>59</v>
       </c>
@@ -1898,7 +1899,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A61" s="2">
         <v>60</v>
       </c>
@@ -1912,7 +1913,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A62" s="2">
         <v>61</v>
       </c>
@@ -1926,12 +1927,12 @@
         <v>44</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A63" s="2">
         <v>62</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="C63" s="2">
         <v>2002</v>
@@ -1940,7 +1941,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A64" s="2">
         <v>63</v>
       </c>
@@ -1954,7 +1955,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A65" s="2">
         <v>64</v>
       </c>
@@ -1968,7 +1969,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A66" s="2">
         <v>65</v>
       </c>
@@ -1982,7 +1983,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A67" s="2">
         <v>66</v>
       </c>
@@ -1996,7 +1997,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A68" s="2">
         <v>67</v>
       </c>
@@ -2010,7 +2011,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A69" s="2">
         <v>68</v>
       </c>
@@ -2024,7 +2025,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A70" s="2">
         <v>69</v>
       </c>
@@ -2038,7 +2039,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A71" s="2">
         <v>70</v>
       </c>
@@ -2052,7 +2053,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A72" s="2">
         <v>71</v>
       </c>
@@ -2066,1197 +2067,1197 @@
         <v>44</v>
       </c>
     </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A73" s="3">
         <v>72</v>
       </c>
       <c r="B73" s="3" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C73" s="3">
         <v>1996</v>
       </c>
       <c r="D73" s="3" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.3">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A74" s="3">
         <v>73</v>
       </c>
       <c r="B74" s="3" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C74" s="3">
         <v>1996</v>
       </c>
       <c r="D74" s="3" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.3">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A75" s="3">
         <v>74</v>
       </c>
       <c r="B75" s="3" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C75" s="3">
         <v>1996</v>
       </c>
       <c r="D75" s="3" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.3">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A76" s="3">
         <v>75</v>
       </c>
       <c r="B76" s="3" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C76" s="3">
         <v>1996</v>
       </c>
       <c r="D76" s="3" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.3">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A77" s="3">
         <v>76</v>
       </c>
       <c r="B77" s="3" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C77" s="3">
         <v>1996</v>
       </c>
       <c r="D77" s="3" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.3">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A78" s="3">
         <v>77</v>
       </c>
       <c r="B78" s="3" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="C78" s="3">
         <v>1996</v>
       </c>
       <c r="D78" s="3" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.3">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A79" s="3">
         <v>78</v>
       </c>
       <c r="B79" s="3" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C79" s="3">
         <v>1996</v>
       </c>
       <c r="D79" s="3" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.3">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A80" s="3">
         <v>79</v>
       </c>
       <c r="B80" s="3" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C80" s="3">
         <v>1996</v>
       </c>
       <c r="D80" s="3" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.3">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A81" s="3">
         <v>80</v>
       </c>
       <c r="B81" s="3" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="C81" s="3">
         <v>1996</v>
       </c>
       <c r="D81" s="3" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.3">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A82" s="3">
         <v>81</v>
       </c>
       <c r="B82" s="3" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="C82" s="3">
         <v>1996</v>
       </c>
       <c r="D82" s="3" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.3">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A83" s="3">
         <v>82</v>
       </c>
       <c r="B83" s="3" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="C83" s="3">
         <v>1996</v>
       </c>
       <c r="D83" s="3" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.3">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A84" s="3">
         <v>83</v>
       </c>
       <c r="B84" s="3" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C84" s="3">
         <v>1996</v>
       </c>
       <c r="D84" s="3" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.3">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A85" s="3">
         <v>84</v>
       </c>
       <c r="B85" s="3" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="C85" s="3">
         <v>1996</v>
       </c>
       <c r="D85" s="3" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.3">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A86" s="3">
         <v>85</v>
       </c>
       <c r="B86" s="3" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C86" s="3">
         <v>1996</v>
       </c>
       <c r="D86" s="3" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.3">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A87" s="3">
         <v>86</v>
       </c>
       <c r="B87" s="3" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C87" s="3">
         <v>1996</v>
       </c>
       <c r="D87" s="3" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.3">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A88" s="3">
         <v>87</v>
       </c>
       <c r="B88" s="3" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C88" s="3">
         <v>1996</v>
       </c>
       <c r="D88" s="3" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.3">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A89" s="3">
         <v>88</v>
       </c>
       <c r="B89" s="3" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C89" s="3">
         <v>1996</v>
       </c>
       <c r="D89" s="3" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.3">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A90" s="3">
         <v>89</v>
       </c>
       <c r="B90" s="3" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C90" s="3">
         <v>1996</v>
       </c>
       <c r="D90" s="3" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.3">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A91" s="3">
         <v>90</v>
       </c>
       <c r="B91" s="3" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C91" s="3">
         <v>1996</v>
       </c>
       <c r="D91" s="3" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.3">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A92" s="4">
         <v>91</v>
       </c>
       <c r="B92" s="4" t="s">
-        <v>166</v>
+        <v>78</v>
       </c>
       <c r="C92" s="4">
         <v>1992</v>
       </c>
       <c r="D92" s="4" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.3">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A93" s="4">
         <v>92</v>
       </c>
       <c r="B93" s="4" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C93" s="4">
         <v>1992</v>
       </c>
       <c r="D93" s="4" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.3">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A94" s="4">
         <v>93</v>
       </c>
       <c r="B94" s="4" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C94" s="4">
         <v>1992</v>
       </c>
       <c r="D94" s="4" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.3">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A95" s="4">
         <v>94</v>
       </c>
       <c r="B95" s="4" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C95" s="4">
         <v>1992</v>
       </c>
       <c r="D95" s="4" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.3">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="96" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A96" s="4">
         <v>95</v>
       </c>
       <c r="B96" s="4" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C96" s="4">
         <v>1992</v>
       </c>
       <c r="D96" s="4" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.3">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A97" s="4">
         <v>96</v>
       </c>
       <c r="B97" s="4" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C97" s="4">
         <v>1992</v>
       </c>
       <c r="D97" s="4" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.3">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="98" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A98" s="4">
         <v>97</v>
       </c>
       <c r="B98" s="4" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C98" s="4">
         <v>1992</v>
       </c>
       <c r="D98" s="4" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.3">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="99" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A99" s="4">
         <v>98</v>
       </c>
       <c r="B99" s="4" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C99" s="4">
         <v>1992</v>
       </c>
       <c r="D99" s="4" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.3">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="100" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A100" s="4">
         <v>99</v>
       </c>
       <c r="B100" s="4" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C100" s="4">
         <v>1992</v>
       </c>
       <c r="D100" s="4" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.3">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="101" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A101" s="4">
         <v>100</v>
       </c>
       <c r="B101" s="4" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C101" s="4">
         <v>1992</v>
       </c>
       <c r="D101" s="4" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.3">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="102" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A102" s="4">
         <v>101</v>
       </c>
       <c r="B102" s="4" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C102" s="4">
         <v>1992</v>
       </c>
       <c r="D102" s="4" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.3">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="103" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A103" s="4">
         <v>102</v>
       </c>
       <c r="B103" s="4" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C103" s="4">
         <v>1992</v>
       </c>
       <c r="D103" s="4" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.3">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="104" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A104" s="2">
         <v>103</v>
       </c>
       <c r="B104" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="C104" s="2">
         <v>1988</v>
       </c>
       <c r="D104" s="2" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.3">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="105" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A105" s="2">
         <v>104</v>
       </c>
       <c r="B105" s="2" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="C105" s="2">
         <v>1988</v>
       </c>
       <c r="D105" s="2" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="106" spans="1:4" x14ac:dyDescent="0.3">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="106" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A106" s="2">
         <v>105</v>
       </c>
       <c r="B106" s="2" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C106" s="2">
         <v>1988</v>
       </c>
       <c r="D106" s="2" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.3">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="107" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A107" s="2">
         <v>106</v>
       </c>
       <c r="B107" s="2" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C107" s="2">
         <v>1988</v>
       </c>
       <c r="D107" s="2" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.3">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="108" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A108" s="2">
         <v>107</v>
       </c>
       <c r="B108" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C108" s="2">
         <v>1988</v>
       </c>
       <c r="D108" s="2" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.3">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="109" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A109" s="2">
         <v>108</v>
       </c>
       <c r="B109" s="2" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="C109" s="2">
         <v>1988</v>
       </c>
       <c r="D109" s="2" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.3">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="110" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A110" s="2">
         <v>109</v>
       </c>
       <c r="B110" s="2" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C110" s="2">
         <v>1988</v>
       </c>
       <c r="D110" s="2" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.3">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="111" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A111" s="2">
         <v>110</v>
       </c>
       <c r="B111" s="2" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="C111" s="2">
         <v>1988</v>
       </c>
       <c r="D111" s="2" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="112" spans="1:4" x14ac:dyDescent="0.3">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="112" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A112" s="2">
         <v>111</v>
       </c>
       <c r="B112" s="2" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="C112" s="2">
         <v>1988</v>
       </c>
       <c r="D112" s="2" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="113" spans="1:4" x14ac:dyDescent="0.3">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="113" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A113" s="2">
         <v>112</v>
       </c>
       <c r="B113" s="2" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="C113" s="2">
         <v>1988</v>
       </c>
       <c r="D113" s="2" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="114" spans="1:4" x14ac:dyDescent="0.3">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="114" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A114" s="2">
         <v>113</v>
       </c>
       <c r="B114" s="2" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="C114" s="2">
         <v>1988</v>
       </c>
       <c r="D114" s="2" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="115" spans="1:4" x14ac:dyDescent="0.3">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="115" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A115" s="2">
         <v>114</v>
       </c>
       <c r="B115" s="2" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C115" s="2">
         <v>1988</v>
       </c>
       <c r="D115" s="2" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="116" spans="1:4" x14ac:dyDescent="0.3">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="116" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A116" s="2">
         <v>115</v>
       </c>
       <c r="B116" s="2" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="C116" s="2">
         <v>1988</v>
       </c>
       <c r="D116" s="2" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="117" spans="1:4" x14ac:dyDescent="0.3">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="117" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A117" s="2">
         <v>116</v>
       </c>
       <c r="B117" s="2" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="C117" s="2">
         <v>1988</v>
       </c>
       <c r="D117" s="2" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="118" spans="1:4" x14ac:dyDescent="0.3">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="118" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A118" s="2">
         <v>117</v>
       </c>
       <c r="B118" s="2" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="C118" s="2">
         <v>1988</v>
       </c>
       <c r="D118" s="2" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="119" spans="1:4" x14ac:dyDescent="0.3">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="119" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A119" s="3">
         <v>118</v>
       </c>
       <c r="B119" s="3" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="C119" s="3">
         <v>1979</v>
       </c>
       <c r="D119" s="3" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="120" spans="1:4" x14ac:dyDescent="0.3">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="120" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A120" s="3">
         <v>119</v>
       </c>
       <c r="B120" s="3" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="C120" s="3">
         <v>1979</v>
       </c>
       <c r="D120" s="3" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="121" spans="1:4" x14ac:dyDescent="0.3">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="121" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A121" s="3">
         <v>120</v>
       </c>
       <c r="B121" s="3" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="C121" s="3">
         <v>1979</v>
       </c>
       <c r="D121" s="3" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="122" spans="1:4" x14ac:dyDescent="0.3">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="122" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A122" s="3">
         <v>121</v>
       </c>
       <c r="B122" s="3" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="C122" s="3">
         <v>1979</v>
       </c>
       <c r="D122" s="3" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="123" spans="1:4" x14ac:dyDescent="0.3">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="123" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A123" s="3">
         <v>122</v>
       </c>
       <c r="B123" s="3" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="C123" s="3">
         <v>1979</v>
       </c>
       <c r="D123" s="3" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="124" spans="1:4" x14ac:dyDescent="0.3">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="124" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A124" s="3">
         <v>123</v>
       </c>
       <c r="B124" s="3" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C124" s="3">
         <v>1979</v>
       </c>
       <c r="D124" s="3" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="125" spans="1:4" x14ac:dyDescent="0.3">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="125" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A125" s="3">
         <v>124</v>
       </c>
       <c r="B125" s="3" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="C125" s="3">
         <v>1979</v>
       </c>
       <c r="D125" s="3" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="126" spans="1:4" x14ac:dyDescent="0.3">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="126" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A126" s="3">
         <v>125</v>
       </c>
       <c r="B126" s="3" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="C126" s="3">
         <v>1979</v>
       </c>
       <c r="D126" s="3" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="127" spans="1:4" x14ac:dyDescent="0.3">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="127" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A127" s="5">
         <v>126</v>
       </c>
       <c r="B127" s="5" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C127" s="5">
         <v>1978</v>
       </c>
       <c r="D127" s="5" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="128" spans="1:4" x14ac:dyDescent="0.3">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="128" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A128" s="5">
         <v>127</v>
       </c>
       <c r="B128" s="5" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="C128" s="5">
         <v>1978</v>
       </c>
       <c r="D128" s="5" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="129" spans="1:4" x14ac:dyDescent="0.3">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="129" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A129" s="5">
         <v>128</v>
       </c>
       <c r="B129" s="5" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C129" s="5">
         <v>1978</v>
       </c>
       <c r="D129" s="5" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="130" spans="1:4" x14ac:dyDescent="0.3">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="130" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A130" s="5">
         <v>129</v>
       </c>
       <c r="B130" s="5" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="C130" s="5">
         <v>1978</v>
       </c>
       <c r="D130" s="5" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="131" spans="1:4" x14ac:dyDescent="0.3">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="131" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A131" s="5">
         <v>130</v>
       </c>
       <c r="B131" s="5" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="C131" s="5">
         <v>1978</v>
       </c>
       <c r="D131" s="5" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="132" spans="1:4" x14ac:dyDescent="0.3">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="132" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A132" s="5">
         <v>131</v>
       </c>
       <c r="B132" s="5" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="C132" s="5">
         <v>1978</v>
       </c>
       <c r="D132" s="5" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="133" spans="1:4" x14ac:dyDescent="0.3">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="133" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A133" s="5">
         <v>132</v>
       </c>
       <c r="B133" s="5" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="C133" s="5">
         <v>1978</v>
       </c>
       <c r="D133" s="5" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="134" spans="1:4" x14ac:dyDescent="0.3">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="134" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A134" s="5">
         <v>133</v>
       </c>
       <c r="B134" s="5" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="C134" s="5">
         <v>1978</v>
       </c>
       <c r="D134" s="5" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="135" spans="1:4" x14ac:dyDescent="0.3">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="135" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A135" s="2">
         <v>134</v>
       </c>
       <c r="B135" s="2" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="C135" s="2">
         <v>1975</v>
       </c>
       <c r="D135" s="2" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="136" spans="1:4" x14ac:dyDescent="0.3">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="136" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A136" s="2">
         <v>135</v>
       </c>
       <c r="B136" s="2" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C136" s="2">
         <v>1975</v>
       </c>
       <c r="D136" s="2" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="137" spans="1:4" x14ac:dyDescent="0.3">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="137" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A137" s="2">
         <v>136</v>
       </c>
       <c r="B137" s="2" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="C137" s="2">
         <v>1975</v>
       </c>
       <c r="D137" s="2" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="138" spans="1:4" x14ac:dyDescent="0.3">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="138" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A138" s="2">
         <v>137</v>
       </c>
       <c r="B138" s="2" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="C138" s="2">
         <v>1975</v>
       </c>
       <c r="D138" s="2" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="139" spans="1:4" x14ac:dyDescent="0.3">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="139" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A139" s="2">
         <v>138</v>
       </c>
       <c r="B139" s="2" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="C139" s="2">
         <v>1975</v>
       </c>
       <c r="D139" s="2" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="140" spans="1:4" x14ac:dyDescent="0.3">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="140" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A140" s="2">
         <v>139</v>
       </c>
       <c r="B140" s="2" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="C140" s="2">
         <v>1975</v>
       </c>
       <c r="D140" s="2" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="141" spans="1:4" x14ac:dyDescent="0.3">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="141" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A141" s="2">
         <v>140</v>
       </c>
       <c r="B141" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C141" s="2">
         <v>1975</v>
       </c>
       <c r="D141" s="2" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="142" spans="1:4" x14ac:dyDescent="0.3">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="142" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A142" s="2">
         <v>141</v>
       </c>
       <c r="B142" s="2" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C142" s="2">
         <v>1975</v>
       </c>
       <c r="D142" s="2" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="143" spans="1:4" x14ac:dyDescent="0.3">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="143" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A143" s="2">
         <v>142</v>
       </c>
       <c r="B143" s="2" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="C143" s="2">
         <v>1975</v>
       </c>
       <c r="D143" s="2" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="144" spans="1:4" x14ac:dyDescent="0.3">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="144" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A144" s="2">
         <v>143</v>
       </c>
       <c r="B144" s="2" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C144" s="2">
         <v>1975</v>
       </c>
       <c r="D144" s="2" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="145" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A145" s="2">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="145" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A145" s="3">
         <v>144</v>
       </c>
-      <c r="B145" s="2" t="s">
-        <v>168</v>
-      </c>
-      <c r="C145" s="2">
+      <c r="B145" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="C145" s="3">
         <v>1975</v>
       </c>
-      <c r="D145" s="2" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="146" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D145" s="3" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="146" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A146" s="3">
         <v>145</v>
       </c>
       <c r="B146" s="3" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="C146" s="3">
         <v>1975</v>
       </c>
       <c r="D146" s="3" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="147" spans="1:4" x14ac:dyDescent="0.3">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="147" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A147" s="3">
         <v>146</v>
       </c>
       <c r="B147" s="3" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="C147" s="3">
         <v>1975</v>
       </c>
       <c r="D147" s="3" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="148" spans="1:4" x14ac:dyDescent="0.3">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="148" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A148" s="3">
         <v>147</v>
       </c>
       <c r="B148" s="3" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="C148" s="3">
         <v>1975</v>
       </c>
       <c r="D148" s="3" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="149" spans="1:4" x14ac:dyDescent="0.3">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="149" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A149" s="3">
         <v>148</v>
       </c>
       <c r="B149" s="3" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="C149" s="3">
         <v>1975</v>
       </c>
       <c r="D149" s="3" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="150" spans="1:4" x14ac:dyDescent="0.3">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="150" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A150" s="3">
         <v>149</v>
       </c>
       <c r="B150" s="3" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="C150" s="3">
         <v>1975</v>
       </c>
       <c r="D150" s="3" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="151" spans="1:4" x14ac:dyDescent="0.3">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="151" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A151" s="3">
         <v>150</v>
       </c>
       <c r="B151" s="3" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="C151" s="3">
         <v>1975</v>
       </c>
       <c r="D151" s="3" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="152" spans="1:4" x14ac:dyDescent="0.3">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="152" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A152" s="3">
         <v>151</v>
       </c>
       <c r="B152" s="3" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="C152" s="3">
         <v>1975</v>
       </c>
       <c r="D152" s="3" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="153" spans="1:4" x14ac:dyDescent="0.3">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="153" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A153" s="3">
         <v>152</v>
       </c>
       <c r="B153" s="3" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="C153" s="3">
         <v>1975</v>
       </c>
       <c r="D153" s="3" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="154" spans="1:4" x14ac:dyDescent="0.3">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="154" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A154" s="3">
         <v>153</v>
       </c>
       <c r="B154" s="3" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="C154" s="3">
         <v>1975</v>
       </c>
       <c r="D154" s="3" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="155" spans="1:4" x14ac:dyDescent="0.3">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="155" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A155" s="3">
         <v>154</v>
       </c>
       <c r="B155" s="3" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="C155" s="3">
         <v>1975</v>
       </c>
       <c r="D155" s="3" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="156" spans="1:4" x14ac:dyDescent="0.3">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="156" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A156" s="3">
         <v>155</v>
       </c>
       <c r="B156" s="3" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C156" s="3">
         <v>1975</v>
       </c>
       <c r="D156" s="3" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="157" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A157" s="3">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="157" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A157" s="5">
         <v>156</v>
       </c>
-      <c r="B157" s="3" t="s">
+      <c r="B157" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="C157" s="3">
+      <c r="C157" s="5">
         <v>1970</v>
       </c>
-      <c r="D157" s="3" t="s">
+      <c r="D157" s="5" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="158" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A158" s="5">
         <v>157</v>
       </c>
@@ -3270,7 +3271,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="159" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A159" s="5">
         <v>158</v>
       </c>
@@ -3284,7 +3285,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="160" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A160" s="5">
         <v>159</v>
       </c>
@@ -3298,7 +3299,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="161" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A161" s="5">
         <v>160</v>
       </c>
@@ -3312,12 +3313,12 @@
         <v>70</v>
       </c>
     </row>
-    <row r="162" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A162" s="5">
         <v>161</v>
       </c>
       <c r="B162" s="5" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C162" s="5">
         <v>1970</v>
@@ -3326,7 +3327,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="163" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A163" s="5">
         <v>162</v>
       </c>
@@ -3340,12 +3341,12 @@
         <v>70</v>
       </c>
     </row>
-    <row r="164" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A164" s="5">
         <v>163</v>
       </c>
       <c r="B164" s="5" t="s">
-        <v>77</v>
+        <v>170</v>
       </c>
       <c r="C164" s="5">
         <v>1970</v>
@@ -3354,7 +3355,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="165" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A165" s="5">
         <v>164</v>
       </c>
@@ -3368,12 +3369,12 @@
         <v>70</v>
       </c>
     </row>
-    <row r="166" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A166" s="5">
         <v>165</v>
       </c>
       <c r="B166" s="5" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C166" s="5">
         <v>1970</v>
@@ -3382,12 +3383,12 @@
         <v>70</v>
       </c>
     </row>
-    <row r="167" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A167" s="5">
         <v>166</v>
       </c>
       <c r="B167" s="5" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C167" s="5">
         <v>1970</v>
@@ -3396,12 +3397,12 @@
         <v>70</v>
       </c>
     </row>
-    <row r="168" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A168" s="5">
         <v>167</v>
       </c>
       <c r="B168" s="5" t="s">
-        <v>79</v>
+        <v>171</v>
       </c>
       <c r="C168" s="5">
         <v>1970</v>
@@ -3423,9 +3424,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ACF1BE34-F7F5-46A0-9E28-C175FFB51C44}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>31</v>
       </c>
@@ -3433,4 +3434,10 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{0cf7ac0a-4681-4823-ab0b-04ef02c5f873}" enabled="1" method="Standard" siteId="{42f7676c-f455-423c-82f6-dc2d99791af7}" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>